<commit_message>
update: excel file and balance
</commit_message>
<xml_diff>
--- a/dataset/custom.xlsx
+++ b/dataset/custom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\matching\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E752A8-A314-4F86-B46F-7B6E620E56B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B6BE2D-1EFA-4117-9DCB-283ECC527706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10060" yWindow="-16110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="매칭결과" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="23">
   <si>
     <t>코트</t>
   </si>
@@ -40,22 +40,63 @@
     <t>팀2_선수2</t>
   </si>
   <si>
+    <t>문민영</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>정지윤</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>김재현</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>박창민</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>안재현</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>정준섭</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>정우용</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>한지윤</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>이영호</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>이희연</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>이영준</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>김신정</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>이도훈</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>서지영</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>이영준</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>문정현</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>김재현</t>
+    <t>강경원</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -63,51 +104,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>이도훈</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>안재현</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>박창민</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>정우용</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>강경원</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>이희연</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>김신정</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>서윤식</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>정준섭</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>정지윤</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>카밀라</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>문민영</t>
+    <t>이희현</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -511,16 +508,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -531,16 +528,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -551,16 +548,16 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -571,16 +568,16 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -591,16 +588,16 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
         <v>15</v>
-      </c>
-      <c r="F6" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -611,16 +608,16 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
         <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -631,16 +628,16 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -651,16 +648,16 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" t="s">
         <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -671,13 +668,13 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s">
         <v>22</v>
@@ -691,16 +688,16 @@
         <v>4</v>
       </c>
       <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
         <v>20</v>
       </c>
-      <c r="D11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" t="s">
-        <v>11</v>
-      </c>
       <c r="F11" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -711,16 +708,16 @@
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -731,16 +728,16 @@
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E13" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F13" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -751,16 +748,16 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
         <v>19</v>
-      </c>
-      <c r="D14" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -771,16 +768,16 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E15" t="s">
         <v>8</v>
       </c>
       <c r="F15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -791,16 +788,16 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E16" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" t="s">
         <v>7</v>
-      </c>
-      <c r="F16" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add: number of time
</commit_message>
<xml_diff>
--- a/dataset/custom.xlsx
+++ b/dataset/custom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\matching\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA489CF-221E-4A70-AA4F-4E5E88742244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267D6F8A-B0AF-46EE-9191-87AFC33F6C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15550" yWindow="-16110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="매칭결과" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="21">
   <si>
     <t>코트</t>
   </si>
@@ -40,76 +40,49 @@
     <t>팀2_선수2</t>
   </si>
   <si>
-    <t>이영호</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>이희연</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <t>서윤식</t>
+  </si>
+  <si>
+    <t>양현철</t>
+  </si>
+  <si>
+    <t>종운동생</t>
+  </si>
+  <si>
+    <t>강경원</t>
+  </si>
+  <si>
+    <t>박종운</t>
+  </si>
+  <si>
+    <t>김양우</t>
+  </si>
+  <si>
+    <t>김종욱</t>
+  </si>
+  <si>
+    <t>김재현</t>
+  </si>
+  <si>
+    <t>박창민</t>
   </si>
   <si>
     <t>안재현</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>정우용</t>
   </si>
   <si>
     <t>이영준</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>이찬호</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>카밀라</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>문정현</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>민규</t>
   </si>
   <si>
     <t>이도훈</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>김종욱</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>김재혁</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>박창민</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>서지영</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>정우용</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>정혜린</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>강경원</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>김재현</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>정지윤</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>김신정</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -518,7 +491,7 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
@@ -532,16 +505,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -552,13 +525,13 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
@@ -572,16 +545,16 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s">
-        <v>16</v>
-      </c>
       <c r="F5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -592,16 +565,16 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
         <v>19</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -612,16 +585,16 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -632,16 +605,16 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -652,16 +625,16 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -672,16 +645,16 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -692,16 +665,16 @@
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -712,16 +685,16 @@
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F12" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -732,13 +705,13 @@
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D13" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E13" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F13" t="s">
         <v>15</v>
@@ -752,16 +725,16 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
         <v>9</v>
       </c>
       <c r="E14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -772,16 +745,16 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E15" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -792,16 +765,16 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" t="s">
         <v>7</v>
-      </c>
-      <c r="E16" t="s">
-        <v>14</v>
-      </c>
-      <c r="F16" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>